<commit_message>
Check lattice vectors matching
</commit_message>
<xml_diff>
--- a/sorted_data.xlsx
+++ b/sorted_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -442,7 +442,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.06736289687278404</v>
+        <v>0.08333465768989165</v>
       </c>
     </row>
     <row r="3">
@@ -452,87 +452,727 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.08075328595125761</v>
+        <v>0.09946736727971436</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>1_1_2_i_57</t>
+          <t>0_2_1_i_63</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.2042574631664717</v>
+        <v>0.2327484917895817</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>1_2_0_i_54</t>
+          <t>1_1_2_i_57</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.2142304541573714</v>
+        <v>0.2529728268152598</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>1_2_2_i_48</t>
+          <t>1_2_0_i_54</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.2324189689615829</v>
+        <v>0.2679468867289865</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>1_2_2_i_49</t>
+          <t>1_0_2_i_62</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.2403639970135119</v>
+        <v>0.269801825326811</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>2_1_2_i_31</t>
+          <t>1_2_2_i_49</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.2409062197744422</v>
+        <v>0.2801578345874216</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>0_2_1_i_63</t>
+          <t>1_2_2_i_48</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.2447083659081823</v>
+        <v>0.2827758347710123</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>2_1_0_i_41</t>
+          <t>0_2_1_i_67</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.2560365038138697</v>
+        <v>0.2858936329895853</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
+          <t>1_2_1_i_50</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0.2933246128032671</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>1_1_1_i_0</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0.2967242948866939</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>2_1_2_i_31</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.3032427265909968</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>1_0_0_i_12</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0.3042968015864624</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>2_1_1_i_36</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0.3135082140095606</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>1_0_1_i_11</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0.3169910453048539</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>1_0_1_i_10</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>0.3195968563968774</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>1_2_1_i_53</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>0.3214206350903534</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>1_2_2_i_45</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>0.3215254619573607</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>2_1_0_i_41</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>0.3230829261258355</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>1_1_0_i_5</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>0.327838477223185</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>2_0_1_i_43</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>0.329221335824247</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
           <t>2_0_1_i_44</t>
         </is>
       </c>
-      <c r="B11" t="n">
-        <v>0.2642692265573601</v>
+      <c r="B23" t="n">
+        <v>0.3352170731680433</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>1_2_2_i_46</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>0.359887157395187</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="inlineStr">
+        <is>
+          <t>0_1_1_i_17</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>0.3672748781563696</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="inlineStr">
+        <is>
+          <t>0_0_1_i_26</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>0.3714397932165489</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="inlineStr">
+        <is>
+          <t>2_1_1_i_39</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>0.3781927467674322</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="inlineStr">
+        <is>
+          <t>1_0_1_i_8</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>0.3804959970493619</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="inlineStr">
+        <is>
+          <t>2_2_1_i_27</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>0.3809857411521007</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="1" t="inlineStr">
+        <is>
+          <t>1_1_1_i_1</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>0.3833865827197461</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="1" t="inlineStr">
+        <is>
+          <t>1_1_1_i_4</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>0.4037137278427529</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="inlineStr">
+        <is>
+          <t>2_1_2_i_34</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>0.4049991195922591</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="inlineStr">
+        <is>
+          <t>2_1_2_i_33</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>0.4068751569151096</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="1" t="inlineStr">
+        <is>
+          <t>0_1_2_i_73</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>0.4090838410500267</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="1" t="inlineStr">
+        <is>
+          <t>0_1_0_i_22</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>0.4133777214670028</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="1" t="inlineStr">
+        <is>
+          <t>2_2_1_i_30</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>0.4165750594412327</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="inlineStr">
+        <is>
+          <t>1_0_2_i_60</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>0.4220844421404924</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="inlineStr">
+        <is>
+          <t>2_0_1_i_42</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>0.4253087934200057</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="1" t="inlineStr">
+        <is>
+          <t>1_2_1_i_52</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>0.4254507350601396</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="1" t="inlineStr">
+        <is>
+          <t>1_1_2_i_59</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>0.4270266857927968</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="inlineStr">
+        <is>
+          <t>2_1_2_i_35</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>0.4270455125291411</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="1" t="inlineStr">
+        <is>
+          <t>1_2_1_i_51</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>0.4295667142483623</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="1" t="inlineStr">
+        <is>
+          <t>1_1_2_i_58</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>0.4304186874503246</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="1" t="inlineStr">
+        <is>
+          <t>1_0_2_i_61</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>0.4346080178930674</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="inlineStr">
+        <is>
+          <t>1_1_0_i_6</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>0.4355846867747353</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="1" t="inlineStr">
+        <is>
+          <t>2_1_0_i_40</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>0.4481678738765252</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="1" t="inlineStr">
+        <is>
+          <t>2_2_1_i_28</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>0.4500802701932677</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="1" t="inlineStr">
+        <is>
+          <t>1_1_1_i_3</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>0.4540999521900165</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="1" t="inlineStr">
+        <is>
+          <t>0_1_2_i_69</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>0.4552792448565163</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="1" t="inlineStr">
+        <is>
+          <t>1_2_2_i_47</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>0.4576325810436055</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="1" t="inlineStr">
+        <is>
+          <t>2_1_2_i_32</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>0.4781116669369158</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="1" t="inlineStr">
+        <is>
+          <t>2_2_1_i_29</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>0.4782481223297911</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="1" t="inlineStr">
+        <is>
+          <t>2_1_1_i_37</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>0.478300930396968</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="1" t="inlineStr">
+        <is>
+          <t>1_1_0_i_7</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>0.4792281241715156</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="1" t="inlineStr">
+        <is>
+          <t>1_2_0_i_55</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>0.4974667367009815</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="1" t="inlineStr">
+        <is>
+          <t>1_2_0_i_56</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>0.5001185576658196</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="1" t="inlineStr">
+        <is>
+          <t>0_2_1_i_64</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>0.5225338896222314</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="1" t="inlineStr">
+        <is>
+          <t>1_1_1_i_2</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>0.5421949034998086</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="1" t="inlineStr">
+        <is>
+          <t>2_1_1_i_38</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>0.5491751026096607</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="1" t="inlineStr">
+        <is>
+          <t>0_2_1_i_65</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>0.5870796524859222</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="1" t="inlineStr">
+        <is>
+          <t>0_0_1_i_25</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>0.5972818211569652</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="1" t="inlineStr">
+        <is>
+          <t>0_1_2_i_68</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>0.6026376070754521</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="1" t="inlineStr">
+        <is>
+          <t>0_1_1_i_15</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>0.6227930948719758</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="1" t="inlineStr">
+        <is>
+          <t>0_0_1_i_23</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>0.6791299443602625</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="1" t="inlineStr">
+        <is>
+          <t>0_1_0_i_19</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>0.7022327719938544</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="1" t="inlineStr">
+        <is>
+          <t>1_0_1_i_9</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>0.7095789102070583</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="1" t="inlineStr">
+        <is>
+          <t>0_1_0_i_20</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>0.7286703861244124</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="1" t="inlineStr">
+        <is>
+          <t>0_1_2_i_72</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>0.7314626222650958</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="1" t="inlineStr">
+        <is>
+          <t>0_1_1_i_16</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>0.7913010972595856</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="1" t="inlineStr">
+        <is>
+          <t>0_1_2_i_70</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>0.8980805252193746</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="1" t="inlineStr">
+        <is>
+          <t>0_1_1_i_14</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>0.931568383822472</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="1" t="inlineStr">
+        <is>
+          <t>0_2_1_i_66</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>0.932954799618955</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="1" t="inlineStr">
+        <is>
+          <t>0_1_2_i_71</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>0.9697666207771185</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="1" t="inlineStr">
+        <is>
+          <t>0_1_1_i_13</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>0.987936926282191</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="1" t="inlineStr">
+        <is>
+          <t>0_0_1_i_24</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>1.109511294044512</v>
       </c>
     </row>
   </sheetData>

</xml_diff>